<commit_message>
Actualizar QA-022 con mediciones de carga y seguimiento de Cloudflare
</commit_message>
<xml_diff>
--- a/Matriz_QA_VAROME_.xlsx
+++ b/Matriz_QA_VAROME_.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="R453056e3cb02435d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz QA" sheetId="2" r:id="Rcf33ba2d3aa0463b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="1" r:id="R944153b5b20549df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz QA" sheetId="2" r:id="R70113111ef6f45fa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,7 +17,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="0%"/>
   </x:numFmts>
-  <x:fonts count="10">
+  <x:fonts count="11">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -70,6 +70,11 @@
     <x:font>
       <x:sz val="9"/>
       <x:color rgb="FF172B3A"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF20384A"/>
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
@@ -148,7 +153,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="81">
+  <x:cellXfs count="86">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -336,6 +341,21 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -669,7 +689,7 @@
       <x:c r="F6" s="7"/>
       <x:c r="G6" s="9" t="n">
         <x:f>B10/C6</x:f>
-        <x:v>0.9666666666666667</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H6" s="9"/>
     </x:row>
@@ -717,7 +737,7 @@
       </x:c>
       <x:c r="B10" s="21" t="n">
         <x:f>COUNTIF('Matriz QA'!J6:J35,A10)</x:f>
-        <x:v>29</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C10" s="18" t="str">
         <x:v>Prueba completada</x:v>
@@ -736,7 +756,7 @@
       </x:c>
       <x:c r="B11" s="22" t="n">
         <x:f>COUNTIF('Matriz QA'!J6:J35,A11)</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C11" s="19" t="str">
         <x:v>Criterio o corrección pendiente</x:v>
@@ -815,7 +835,7 @@
     </x:row>
     <x:row r="17" ht="60" customHeight="1">
       <x:c r="A17" s="38" t="str">
-        <x:v>Pendiente: definir criterio de carga (QA-022). Favicon y Región corregidos y validados. QA-016 y QA-017 conservan resultado histórico con respaldo técnico pendiente.</x:v>
+        <x:v>30 casos con estado Aprobado. QA-016 y QA-017 conservan resultado histórico con respaldo técnico pendiente. Tres advertencias de Cloudflare siguen abiertas para seguimiento.</x:v>
       </x:c>
       <x:c r="B17" s="35"/>
       <x:c r="C17" s="35"/>
@@ -826,34 +846,36 @@
       <x:c r="H17" s="80" t="str"/>
     </x:row>
     <x:row r="18" ht="28" customHeight="1">
-      <x:c r="A18" s="39"/>
-      <x:c r="B18" s="36"/>
-      <x:c r="C18" s="36"/>
-      <x:c r="D18" s="36"/>
-      <x:c r="E18" s="44" t="str"/>
-      <x:c r="F18" s="44" t="str"/>
-      <x:c r="G18" s="44" t="str"/>
-      <x:c r="H18" s="44" t="str"/>
+      <x:c r="A18" s="81" t="str">
+        <x:v>Cloudflare: Protected Audience API, StorageType.persistent y Fenced Frame API obsoletos. Origen confirmado por usuaria: /cdn-cgi/challenge-platform/scripts/jsd/main.js. Evidencias 29–31 en GitHub.</x:v>
+      </x:c>
+      <x:c r="B18" s="82"/>
+      <x:c r="C18" s="82"/>
+      <x:c r="D18" s="82"/>
+      <x:c r="E18" s="83" t="str"/>
+      <x:c r="F18" s="83" t="str"/>
+      <x:c r="G18" s="83" t="str"/>
+      <x:c r="H18" s="83" t="str"/>
     </x:row>
     <x:row r="19" ht="28" customHeight="1">
-      <x:c r="A19" s="39"/>
-      <x:c r="B19" s="36"/>
-      <x:c r="C19" s="36"/>
-      <x:c r="D19" s="36"/>
-      <x:c r="E19" s="44" t="str"/>
-      <x:c r="F19" s="44" t="str"/>
-      <x:c r="G19" s="44" t="str"/>
-      <x:c r="H19" s="44" t="str"/>
+      <x:c r="A19" s="81"/>
+      <x:c r="B19" s="82"/>
+      <x:c r="C19" s="82"/>
+      <x:c r="D19" s="82"/>
+      <x:c r="E19" s="83" t="str"/>
+      <x:c r="F19" s="83" t="str"/>
+      <x:c r="G19" s="83" t="str"/>
+      <x:c r="H19" s="83" t="str"/>
     </x:row>
     <x:row r="20" ht="28" customHeight="1">
-      <x:c r="A20" s="40"/>
-      <x:c r="B20" s="37"/>
-      <x:c r="C20" s="37"/>
-      <x:c r="D20" s="37"/>
-      <x:c r="E20" s="44" t="str"/>
-      <x:c r="F20" s="44" t="str"/>
-      <x:c r="G20" s="44" t="str"/>
-      <x:c r="H20" s="44" t="str"/>
+      <x:c r="A20" s="84"/>
+      <x:c r="B20" s="85"/>
+      <x:c r="C20" s="85"/>
+      <x:c r="D20" s="85"/>
+      <x:c r="E20" s="83" t="str"/>
+      <x:c r="F20" s="83" t="str"/>
+      <x:c r="G20" s="83" t="str"/>
+      <x:c r="H20" s="83" t="str"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="44"/>
@@ -910,6 +932,7 @@
     <x:mergeCell ref="A16:H16"/>
     <x:mergeCell ref="A22:H22"/>
     <x:mergeCell ref="A17:H17"/>
+    <x:mergeCell ref="A18:H20"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1798,7 +1821,7 @@
         <x:v>Corrección publicada en versión 11: cobertura a lo largo de Chile y redacción técnica ajustada.</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="97.19999694824219" hidden="0" customHeight="1">
+    <x:row r="27" ht="194.39999389648438" hidden="0" customHeight="1">
       <x:c r="A27" s="74" t="str">
         <x:v>QA-022</x:v>
       </x:c>
@@ -1809,33 +1832,36 @@
         <x:v>Carga inicial</x:v>
       </x:c>
       <x:c r="D27" s="71" t="str">
-        <x:v>Chrome; Disable cache activado; No throttling; conexión del equipo de prueba</x:v>
+        <x:v>Chrome incógnito; Disable cache activado; No throttling; conexión del equipo de prueba.</x:v>
       </x:c>
       <x:c r="E27" s="71" t="str">
         <x:v>Recargar tres veces y registrar Load en Network</x:v>
       </x:c>
       <x:c r="F27" s="71" t="str">
-        <x:v>Registrar Load; umbral de aceptación pendiente de definir</x:v>
+        <x:v>Load ≤ 5 segundos en cada una de tres recargas. Criterio adoptado para esta prueba del proyecto.</x:v>
       </x:c>
       <x:c r="G27" s="71" t="str">
-        <x:v>09-10-2026: Load 4,67 s; 3,54 s; 4,64 s. Promedio 4,28 s; mediana 4,64 s.</x:v>
+        <x:v>23-10-2026: Load 0,284 s; 2,36 s; 2,31 s. Promedio 1,6513 s (1,65 s); mediana 2,31 s. Las tres mediciones cumplen ≤ 5 s.</x:v>
       </x:c>
       <x:c r="H27" s="71" t="str">
         <x:v>https://github.com/mduque142-pixel/mduque142-pixel.github.io/blob/main/evidencias-qa/evidencias-qa-varome/qa-varome-20-carga-01.png
 https://github.com/mduque142-pixel/mduque142-pixel.github.io/blob/main/evidencias-qa/evidencias-qa-varome/qa-varome-20-carga-02.png
-https://github.com/mduque142-pixel/mduque142-pixel.github.io/blob/main/evidencias-qa/evidencias-qa-varome/qa-varome-20-carga-03.png</x:v>
+https://github.com/mduque142-pixel/mduque142-pixel.github.io/blob/main/evidencias-qa/evidencias-qa-varome/qa-varome-20-carga-03.png
+https://github.com/mduque142-pixel/mduque142-pixel.github.io/blob/main/evidencias-qa/evidencias-qa-varome/qa-varome-32-carga-01.png
+https://github.com/mduque142-pixel/mduque142-pixel.github.io/blob/main/evidencias-qa/evidencias-qa-varome/qa-varome-33-carga-02.png
+https://github.com/mduque142-pixel/mduque142-pixel.github.io/blob/main/evidencias-qa/evidencias-qa-varome/qa-varome-34-carga-03.png</x:v>
       </x:c>
       <x:c r="I27" s="77" t="str">
         <x:v>Baja</x:v>
       </x:c>
       <x:c r="J27" s="77" t="str">
-        <x:v>Pendiente</x:v>
+        <x:v>Aprobado</x:v>
       </x:c>
       <x:c r="K27" s="77" t="str">
         <x:v>QA VAROME</x:v>
       </x:c>
       <x:c r="L27" s="71" t="str">
-        <x:v>Medición realizada; aprobación pendiente de criterio. No equivale a Core Web Vitals. Referencia histórica del 05-10-2026 (métrica no precisada): La página principal cargó de forma estable en tres repeticiones: 2.074 s, 1.191 s y 0.398 s. Promedio 1.221 s y mediana 1.191 s, sin errores propios del sitio.</x:v>
+        <x:v>23-10-2026: evidencias 32–34 registradas en GitHub, confirmado por usuaria. Aprobación limitada a tres recargas y condiciones indicadas; no equivale a Core Web Vitals ni prueba de usuarios concurrentes. Histórico 09-10-2026: Load 4,67 s; 3,54 s; 4,64 s (promedio 4,28 s), entonces sin criterio definido. Histórico 05-10-2026: 2,074 s; 1,191 s; 0,398 s, métrica no precisada.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="43.20000076293945" hidden="0" customHeight="1">

</xml_diff>